<commit_message>
update excel importation templates
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_4g.xlsx
+++ b/backend/templates/template_cell_4g.xlsx
@@ -584,21 +584,21 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="26" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
-    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
-    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -699,7 +699,7 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Baseband</t>
+          <t>Chung anten</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -734,42 +734,42 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Chung anten</t>
+          <t>EnodeB ID</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>EnodeB ID</t>
+          <t>EARFCN</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>EARFCN</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>PCI</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>PCI</t>
+          <t>Root Sequence ID</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Root Sequence ID</t>
+          <t>Bandwitdh</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Bandwitdh</t>
+          <t>ECI</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>ECI</t>
+          <t>OSS</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,11 @@
       </c>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>4G only</t>
+        </is>
+      </c>
       <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="n"/>
       <c r="W2" s="2" t="inlineStr">
@@ -836,17 +840,13 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>4G</t>
-        </is>
-      </c>
+      <c r="AA2" s="2" t="n"/>
       <c r="AB2" s="2" t="n"/>
       <c r="AC2" s="2" t="n"/>
-      <c r="AD2" s="2" t="n"/>
-      <c r="AE2" s="2" t="n">
+      <c r="AD2" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
       <c r="AH2" s="2" t="n"/>
@@ -36817,7 +36817,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AH1"/>
-  <dataValidations count="14">
+  <dataValidations count="13">
     <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"MB,MT,MN"</formula1>
     </dataValidation>
@@ -36850,13 +36850,10 @@
     <dataValidation sqref="S2:S1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>'_Lookups'!$C$2:$C$83</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
-      <formula1>"2x2,4x4,8x8"</formula1>
+    <dataValidation sqref="T2:T1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"4G only,3G4G,2G3G4G,4G5G,3G4G5G"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
-      <formula1>"4G,2G/4G,3G/4G,2G/3G/4G,4G/5G"</formula1>
-    </dataValidation>
-    <dataValidation sqref="AE2:AE1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="PCI không hợp lệ" error="PCI phải trong khoảng 0 – 503" type="whole" operator="between">
+    <dataValidation sqref="AD2:AD1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="PCI không hợp lệ" error="PCI phải trong khoảng 0 – 503" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>503</formula2>
     </dataValidation>
@@ -36875,7 +36872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -37160,107 +37157,95 @@
       </c>
       <c r="C26" s="9" t="inlineStr"/>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Tinh / Phuong xa để trống</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>→ Tự động điền theo 6 ký tự đầu của Cell Name (khớp cột ky_tu_1_6 trong danh mục Tỉnh/Xã/Phường). Ví dụ: HNIHKM44DI4DA → HNIHKM</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Tinh / Phuong xa đã có giá trị</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>→ Giữ nguyên giá trị đã nhập, KHÔNG tự động điền</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Không tìm thấy mã 6 ký tự</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>→ Tinh / Phuong xa để trống (không phải lỗi – các cột này KHÔNG bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>MÔ TẢ CÁC CỘT</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Tên cột</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Mô tả / Hướng dẫn</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>Bắt buộc</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Mien</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Miền: MB / MT / MN</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Tinh</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Tỉnh / Thành phố – chọn từ danh sách</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>Phuong xa</t>
-        </is>
-      </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>Phường / Xã – chọn từ danh sách</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Site Name</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Tên site – bắt buộc, phải khớp với site đã có</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>✔ Bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Site Name Old</t>
+          <t>Tinh</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Tên site cũ – điền khi site vừa đổi tên</t>
+          <t>Tỉnh / Thành phố – chọn từ danh sách. KHÔNG bắt buộc – để trống thì hệ thống tự điền theo 6 ký tự đầu của Cell Name (khớp cột ky_tu_1_6 trong danh mục Tỉnh/Xã/Phường); đã nhập thì giữ nguyên</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -37270,116 +37255,116 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Cell Name</t>
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Phuong xa</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Tên cell – bắt buộc, duy nhất trong site</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
+          <t>Phường / Xã – chọn từ danh sách. KHÔNG bắt buộc – để trống thì hệ thống tự điền theo 6 ký tự đầu của Cell Name (khớp cột ky_tu_1_6 trong danh mục Tỉnh/Xã/Phường); đã nhập thì giữ nguyên</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Site Name</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Tên site – bắt buộc, phải khớp với site đã có</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>✔ Bắt buộc</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>Cell Name Old</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Tên cell cũ – điền khi cell vừa đổi tên</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
+          <t>Site Name Old</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Tên site cũ – điền khi site vừa đổi tên</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Cell Name</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Tên cell – bắt buộc, duy nhất trong site (vd: HNIHKM44DI4DA)</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>✔ Bắt buộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Cell Name Old</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Tên cell cũ – điền khi cell vừa đổi tên</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
           <t>Cell VIP</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>Mức độ VIP: VIP hoặc VVIP</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>MORAN</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>MORAN: VNPT HOST hoặc MBF HOST</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Lat</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Latitude – phải trong 8.33–23.39</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>✔ Bắt buộc</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Longitude – phải trong 102.14–109.47</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>✔ Bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>Vung phu song</t>
+          <t>MORAN</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Vùng phủ sóng: Indoor hoặc Outdoor</t>
+          <t>MORAN: VNPT HOST hoặc MBF HOST</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -37391,12 +37376,12 @@
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Vendor</t>
+          <t>Lat</t>
         </is>
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>Hãng thiết bị – bắt buộc, chọn từ danh sách</t>
+          <t>Latitude – phải trong 8.33–23.39</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -37408,12 +37393,12 @@
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Do cao anten</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>Độ cao anten – bắt buộc (số hoặc chuỗi, vd: 28 hoặc IBC)</t>
+          <t>Longitude – phải trong 102.14–109.47</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
@@ -37423,31 +37408,31 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Azimuth</t>
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>Vung phu song</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Góc phương vị – bắt buộc (số hoặc chuỗi, vd: 120 hoặc IBC)</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>✔ Bắt buộc</t>
+          <t>Vùng phủ sóng: Indoor hoặc Outdoor</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>M-tilt</t>
+          <t>Vendor</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Mechanical tilt – bắt buộc (số hoặc chuỗi, vd: 2 hoặc IBC)</t>
+          <t>Hãng thiết bị – bắt buộc, chọn từ danh sách</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -37459,80 +37444,80 @@
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
+          <t>Do cao anten</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>Độ cao anten – bắt buộc (số hoặc chuỗi, vd: 28 hoặc IBC)</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>✔ Bắt buộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Azimuth</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>Góc phương vị – bắt buộc (số hoặc chuỗi, vd: 120 hoặc IBC)</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>✔ Bắt buộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>M-tilt</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>Mechanical tilt – bắt buộc (số hoặc chuỗi, vd: 2 hoặc IBC)</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>✔ Bắt buộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
           <t>E-Tilt</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>Electrical tilt – bắt buộc (số hoặc chuỗi, vd: 4 hoặc IBC)</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>✔ Bắt buộc</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t>Total Tilt</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>Tổng tilt (số hoặc chuỗi, tự tính hoặc để trống)</t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
-        <is>
-          <t>Loai Anten</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>Loại anten – chọn từ danh sách antenna</t>
-        </is>
-      </c>
-      <c r="C48" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>Baseband</t>
-        </is>
-      </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>Tên thiết bị baseband</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="inlineStr">
-        <is>
-          <t>Tùy chọn</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>Total Tilt</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>Tên thiết bị RF</t>
+          <t>Tổng tilt (số hoặc chuỗi, tự tính hoặc để trống)</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -37544,12 +37529,12 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>Cell ID</t>
+          <t>Loai Anten</t>
         </is>
       </c>
       <c r="B51" s="13" t="inlineStr">
         <is>
-          <t>Cell ID (chuỗi hoặc số)</t>
+          <t>Loại anten – chọn từ danh sách antenna</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
@@ -37561,12 +37546,12 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>MIMO</t>
+          <t>Chung anten</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình MIMO: 2x2 / 4x4 / 8x8</t>
+          <t>Chung anten – chọn từ danh sách: 4G only, 3G4G, 2G3G4G, 4G5G, 3G4G5G</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
@@ -37578,12 +37563,12 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>Cell max power (dBm)</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>Công suất tối đa cell (dBm)</t>
+          <t>Tên thiết bị RF</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -37595,12 +37580,12 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>BBUname</t>
+          <t>Cell ID</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
-          <t>Tên BBU</t>
+          <t>Cell ID (chuỗi hoặc số)</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
@@ -37612,12 +37597,12 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>Cell status (at dump time)</t>
+          <t>MIMO</t>
         </is>
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>Trạng thái cell tại thời điểm dump</t>
+          <t>Cấu hình MIMO – nhập tự do (vd: 2x2, 4x4, 8x8, 32T32R)</t>
         </is>
       </c>
       <c r="C55" s="14" t="inlineStr">
@@ -37629,12 +37614,12 @@
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>Chung anten</t>
+          <t>Cell max power (dBm)</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
-          <t>Chung anten 4G: 4G / 2G/4G / 3G/4G / 2G/3G/4G / 4G/5G</t>
+          <t>Công suất tối đa cell (dBm)</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -37646,12 +37631,12 @@
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>EnodeB ID</t>
+          <t>BBUname</t>
         </is>
       </c>
       <c r="B57" s="13" t="inlineStr">
         <is>
-          <t>eNodeB ID</t>
+          <t>Tên BBU</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -37663,12 +37648,12 @@
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>EARFCN</t>
+          <t>Cell status (at dump time)</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
-          <t>E-UTRA Absolute Radio Frequency Channel Number</t>
+          <t>Trạng thái cell tại thời điểm dump</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
@@ -37680,12 +37665,12 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>EnodeB ID</t>
         </is>
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
-          <t>Tracking Area Code</t>
+          <t>eNodeB ID</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -37697,12 +37682,12 @@
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>PCI</t>
+          <t>EARFCN</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>Physical Cell Identity 0–503</t>
+          <t>E-UTRA Absolute Radio Frequency Channel Number</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
@@ -37714,12 +37699,12 @@
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>Root Sequence ID</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>Root Sequence Index</t>
+          <t>Tracking Area Code</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
@@ -37731,12 +37716,12 @@
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>Bandwitdh</t>
+          <t>PCI</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
         <is>
-          <t>Bandwidth (MHz) – ví dụ: 5, 10, 15, 20</t>
+          <t>Physical Cell Identity 0–503</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
@@ -37748,15 +37733,66 @@
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
+          <t>Root Sequence ID</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Root Sequence Index</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>Bandwitdh</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Bandwidth (MHz) – ví dụ: 5, 10, 15, 20</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
           <t>ECI</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B65" s="13" t="inlineStr">
         <is>
           <t>E-UTRAN Cell Identifier</t>
         </is>
       </c>
-      <c r="C63" s="14" t="inlineStr">
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Tùy chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>OSS</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Hệ thống OSS nguồn dữ liệu – nhập tự do</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>Tùy chọn</t>
         </is>
@@ -37764,9 +37800,9 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>

</xml_diff>